<commit_message>
Update CCA TotMktVal, update column note
</commit_message>
<xml_diff>
--- a/input/community_cohort_inputs_2026_DAonly.xlsx
+++ b/input/community_cohort_inputs_2026_DAonly.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amcadams\GitHub\community-cohort-tool\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDDD1FB0-9167-465F-9EE3-3ABE4E33E4F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D94A79DE-53A4-4BF0-8C6C-E3AB0144875F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26670" yWindow="6255" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14730" yWindow="-16455" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FACTORS_MUNI" sheetId="1" r:id="rId1"/>
@@ -400,7 +400,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve"> Total market value, calculated from 2021 county assessor data. For each Chicago PIN, total market value is calculated by multiplying total assessed value by a factor, depending on the parcel's class. Factors are as follows: 10x for classes 100-399 &amp; 600-999; 5x for classes 400-499; and 4x for classes 500-599.
+          <t xml:space="preserve"> Total market value, calculated from 2023 Cook County Assessor's Office data. For each Chicago PIN, total market value is calculated by multiplying total assessed value by a factor, depending on the parcel's class. Factors are generally as follows: 10x for classes 100-399 &amp; 600-999; 5x for classes 400-499; and 4x for classes 500-599. For more information see the CCAO's website: https://www.cookcountyassessoril.gov/classifications-real-property
 </t>
         </r>
         <r>
@@ -422,7 +422,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve"> Chicago is reassessed on a triennial basis, with the most recent assessment being done in 2021. This variable can next be updated with the 2023 assessor data.</t>
+          <t xml:space="preserve"> Chicago is reassessed on a triennial basis, with the most recent assessment being done in 2023. This variable can next be updated with the 2025 assessor data.</t>
         </r>
       </text>
     </comment>
@@ -1898,11 +1898,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.00000"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="30" x14ac:knownFonts="1">
     <font>
@@ -2520,7 +2519,7 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2542,17 +2541,16 @@
     <xf numFmtId="1" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="42" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="19" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="21" fillId="33" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="16" fillId="33" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="21" fillId="33" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="21" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="21" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="21" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="21" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2925,19 +2923,19 @@
       <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="30" t="s">
+      <c r="D1" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="25" t="s">
+      <c r="G1" s="28" t="s">
         <v>379</v>
       </c>
       <c r="H1" s="17" t="s">
@@ -13991,11 +13989,11 @@
         <v>12051912</v>
       </c>
       <c r="I258" s="4">
-        <f t="shared" ref="I258:I321" si="21">H258/C258</f>
+        <f t="shared" ref="I258:I285" si="21">H258/C258</f>
         <v>38627.923076923078</v>
       </c>
       <c r="J258" s="8">
-        <f t="shared" ref="J258:J321" si="22">LN(I258)</f>
+        <f t="shared" ref="J258:J285" si="22">LN(I258)</f>
         <v>10.561730689703523</v>
       </c>
       <c r="K258" s="8">
@@ -15191,7 +15189,7 @@
     <col min="4" max="4" width="13.6640625" style="15" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.44140625" style="16" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" style="16" customWidth="1"/>
-    <col min="7" max="7" width="19" style="23" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19" style="22" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.6640625" style="8" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.109375" style="8"/>
     <col min="10" max="10" width="15.6640625" style="8" bestFit="1" customWidth="1"/>
@@ -15204,19 +15202,19 @@
       <c r="B1" s="14" t="s">
         <v>375</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="29" t="s">
         <v>379</v>
       </c>
-      <c r="E1" s="27" t="s">
+      <c r="E1" s="30" t="s">
         <v>378</v>
       </c>
-      <c r="F1" s="29" t="s">
+      <c r="F1" s="25" t="s">
         <v>377</v>
       </c>
-      <c r="G1" s="22" t="s">
+      <c r="G1" s="21" t="s">
         <v>7</v>
       </c>
       <c r="H1" s="7" t="s">
@@ -15231,2780 +15229,2780 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>356</v>
+        <v>298</v>
       </c>
       <c r="C2" s="19">
-        <v>60915.74</v>
+        <v>86513.02</v>
       </c>
       <c r="D2" s="15">
-        <v>0.29557057596893649</v>
+        <v>0.1205471526572444</v>
       </c>
       <c r="E2">
-        <v>3945507288</v>
+        <v>3517069214.2389002</v>
       </c>
       <c r="F2">
-        <v>54173</v>
-      </c>
-      <c r="G2" s="23">
+        <v>45538</v>
+      </c>
+      <c r="G2" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E2/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F2)</f>
-        <v>30653.077032788016</v>
+        <v>31506.959497000469</v>
       </c>
       <c r="H2" s="8">
-        <f t="shared" ref="H2:H33" si="0">LN(G2)</f>
-        <v>10.330488328912244</v>
+        <f>LN(G2)</f>
+        <v>10.357963736823583</v>
       </c>
       <c r="I2" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J2" s="8">
-        <f t="shared" ref="J2:J33" si="1">LN(C2)</f>
-        <v>11.017246876789907</v>
+        <f>LN(C2)</f>
+        <v>11.36805020182415</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>2</v>
+        <v>57</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>371</v>
+        <v>299</v>
       </c>
       <c r="C3" s="19">
-        <v>70823.37</v>
+        <v>67012.2</v>
       </c>
       <c r="D3" s="15">
-        <v>5.750628873732528E-2</v>
+        <v>9.270216962524655E-2</v>
       </c>
       <c r="E3">
-        <v>5358863377.8789196</v>
+        <v>995573111.824772</v>
       </c>
       <c r="F3">
-        <v>78373</v>
-      </c>
-      <c r="G3" s="23">
+        <v>13414</v>
+      </c>
+      <c r="G3" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E3/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F3)</f>
-        <v>29650.652861522729</v>
+        <v>30833.97000619163</v>
       </c>
       <c r="H3" s="8">
-        <f t="shared" si="0"/>
-        <v>10.29723942312183</v>
+        <f>LN(G3)</f>
+        <v>10.33637228346868</v>
       </c>
       <c r="I3" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J3" s="8">
-        <f t="shared" si="1"/>
-        <v>11.167944309961589</v>
+        <f>LN(C3)</f>
+        <v>11.112629971349051</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>363</v>
+        <v>300</v>
       </c>
       <c r="C4" s="19">
-        <v>70066.83</v>
+        <v>45340.34</v>
       </c>
       <c r="D4" s="15">
-        <v>0</v>
+        <v>0.21713462922966162</v>
       </c>
       <c r="E4">
-        <v>6215659728</v>
-      </c>
-      <c r="F4">
-        <v>56344</v>
-      </c>
-      <c r="G4" s="23">
+        <v>1390091360</v>
+      </c>
+      <c r="F4" s="20">
+        <v>13885</v>
+      </c>
+      <c r="G4" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E4/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F4)</f>
-        <v>39087.116899312306</v>
+        <v>36614.690314284497</v>
       </c>
       <c r="H4" s="8">
-        <f t="shared" si="0"/>
-        <v>10.573548200613168</v>
+        <f>LN(G4)</f>
+        <v>10.508204813567405</v>
       </c>
       <c r="I4" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J4" s="8">
-        <f t="shared" si="1"/>
-        <v>11.157204779867387</v>
+        <f>LN(C4)</f>
+        <v>10.721952422930624</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>337</v>
+        <v>301</v>
       </c>
       <c r="C5" s="19">
-        <v>92490.48</v>
+        <v>82235.360000000001</v>
       </c>
       <c r="D5" s="15">
-        <v>0</v>
+        <v>0.30595162781643875</v>
       </c>
       <c r="E5">
-        <v>5335063217</v>
+        <v>2615780810.5645399</v>
       </c>
       <c r="F5">
-        <v>41651</v>
-      </c>
-      <c r="G5" s="23">
+        <v>42007</v>
+      </c>
+      <c r="G5" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E5/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F5)</f>
-        <v>43086.131870496196</v>
+        <v>28166.614389520677</v>
       </c>
       <c r="H5" s="8">
-        <f t="shared" si="0"/>
-        <v>10.670956457968146</v>
+        <f>LN(G5)</f>
+        <v>10.245892668682085</v>
       </c>
       <c r="I5" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J5" s="8">
-        <f t="shared" si="1"/>
-        <v>11.434860999285082</v>
+        <f>LN(C5)</f>
+        <v>11.317340658863849</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>5</v>
+        <v>71</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>348</v>
+        <v>302</v>
       </c>
       <c r="C6" s="19">
-        <v>145659.34</v>
+        <v>47170.47</v>
       </c>
       <c r="D6" s="15">
-        <v>0</v>
+        <v>0.59438923303177504</v>
       </c>
       <c r="E6">
-        <v>7458343008.5430002</v>
+        <v>1834998656</v>
       </c>
       <c r="F6">
-        <v>36014</v>
-      </c>
-      <c r="G6" s="23">
+        <v>43779</v>
+      </c>
+      <c r="G6" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E6/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F6)</f>
-        <v>60862.464635562719</v>
+        <v>23622.724356361257</v>
       </c>
       <c r="H6" s="8">
-        <f t="shared" si="0"/>
-        <v>11.01637191943616</v>
+        <f>LN(G6)</f>
+        <v>10.069964424182269</v>
       </c>
       <c r="I6" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J6" s="8">
-        <f t="shared" si="1"/>
-        <v>11.88902588666182</v>
+        <f>LN(C6)</f>
+        <v>10.761523340188811</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>335</v>
+        <v>303</v>
       </c>
       <c r="C7" s="19">
-        <v>105498.97</v>
+        <v>47532.57</v>
       </c>
       <c r="D7" s="15">
-        <v>0</v>
+        <v>0.49213417981088892</v>
       </c>
       <c r="E7">
-        <v>20148584267.721901</v>
+        <v>4682392586.92484</v>
       </c>
       <c r="F7">
-        <v>102827</v>
-      </c>
-      <c r="G7" s="23">
+        <v>97452</v>
+      </c>
+      <c r="G7" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E7/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F7)</f>
-        <v>58353.891757258825</v>
+        <v>24991.835746419685</v>
       </c>
       <c r="H7" s="8">
-        <f t="shared" si="0"/>
-        <v>10.974281332273069</v>
+        <f>LN(G7)</f>
+        <v>10.126304480371484</v>
       </c>
       <c r="I7" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J7" s="8">
-        <f t="shared" si="1"/>
-        <v>11.566456468817425</v>
+        <f>LN(C7)</f>
+        <v>10.769170439259247</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>336</v>
+        <v>304</v>
       </c>
       <c r="C8" s="19">
-        <v>137914.1</v>
+        <v>57862.6</v>
       </c>
       <c r="D8" s="15">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>20868022993.062698</v>
-      </c>
-      <c r="F8">
-        <v>67987</v>
-      </c>
-      <c r="G8" s="23">
+        <v>555002732</v>
+      </c>
+      <c r="F8" s="20">
+        <v>9024</v>
+      </c>
+      <c r="G8" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E8/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F8)</f>
-        <v>83327.734503740736</v>
+        <v>27995.361411261059</v>
       </c>
       <c r="H8" s="8">
-        <f t="shared" si="0"/>
-        <v>11.330536719964085</v>
+        <f>LN(G8)</f>
+        <v>10.239794111550031</v>
       </c>
       <c r="I8" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J8" s="8">
-        <f t="shared" si="1"/>
-        <v>11.834386306560223</v>
+        <f>LN(C8)</f>
+        <v>10.965826513573072</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>344</v>
+        <v>305</v>
       </c>
       <c r="C9" s="19">
-        <v>124208.23</v>
+        <v>93915.78</v>
       </c>
       <c r="D9" s="15">
         <v>0</v>
       </c>
       <c r="E9">
-        <v>132811651780.245</v>
+        <v>3871744648.01126</v>
       </c>
       <c r="F9">
-        <v>107331</v>
-      </c>
-      <c r="G9" s="23">
+        <v>35533</v>
+      </c>
+      <c r="G9" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E9/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F9)</f>
-        <v>292681.35086524813</v>
+        <v>38589.691639060991</v>
       </c>
       <c r="H9" s="8">
-        <f t="shared" si="0"/>
-        <v>12.586839756489734</v>
+        <f>LN(G9)</f>
+        <v>10.560740463804247</v>
       </c>
       <c r="I9" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J9" s="8">
-        <f t="shared" si="1"/>
-        <v>11.729714710376324</v>
+        <f>LN(C9)</f>
+        <v>11.450153702195557</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>320</v>
+        <v>306</v>
       </c>
       <c r="C10" s="19">
-        <v>128066.04</v>
+        <v>68284.210000000006</v>
       </c>
       <c r="D10" s="15">
-        <v>0</v>
+        <v>0.4069716831378975</v>
       </c>
       <c r="E10">
-        <v>1738199600</v>
+        <v>3906307642.5862598</v>
       </c>
       <c r="F10">
-        <v>11558</v>
-      </c>
-      <c r="G10" s="23">
+        <v>72088</v>
+      </c>
+      <c r="G10" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E10/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F10)</f>
-        <v>48103.544483575242</v>
+        <v>26362.442345131214</v>
       </c>
       <c r="H10" s="8">
-        <f t="shared" si="0"/>
-        <v>10.781111143266106</v>
+        <f>LN(G10)</f>
+        <v>10.179695637781554</v>
       </c>
       <c r="I10" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J10" s="8">
-        <f t="shared" si="1"/>
-        <v>11.760301347351763</v>
+        <f>LN(C10)</f>
+        <v>11.131433832886929</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>10</v>
+        <v>72</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>351</v>
+        <v>307</v>
       </c>
       <c r="C11" s="19">
-        <v>110554.42</v>
+        <v>132096.54</v>
       </c>
       <c r="D11" s="15">
-        <v>0.3766284625225178</v>
+        <v>0</v>
       </c>
       <c r="E11">
-        <v>4738453822</v>
-      </c>
-      <c r="F11" s="20">
-        <v>39840</v>
-      </c>
-      <c r="G11" s="23">
+        <v>2170458788</v>
+      </c>
+      <c r="F11">
+        <v>19521</v>
+      </c>
+      <c r="G11" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E11/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F11)</f>
-        <v>41026.801682760772</v>
+        <v>39086.135609118603</v>
       </c>
       <c r="H11" s="8">
-        <f t="shared" si="0"/>
-        <v>10.621980831697474</v>
+        <f>LN(G11)</f>
+        <v>10.573523095090184</v>
       </c>
       <c r="I11" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J11" s="8">
-        <f t="shared" si="1"/>
-        <v>11.613263167394976</v>
+        <f>LN(C11)</f>
+        <v>11.791288297888816</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>11</v>
+        <v>60</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>333</v>
+        <v>308</v>
       </c>
       <c r="C12" s="19">
-        <v>96869.59</v>
+        <v>74609.509999999995</v>
       </c>
       <c r="D12" s="15">
-        <v>0.37648764113518463</v>
+        <v>7.6879710402943446E-2</v>
       </c>
       <c r="E12">
-        <v>2760477311.1213899</v>
-      </c>
-      <c r="F12">
-        <v>26649</v>
-      </c>
-      <c r="G12" s="23">
+        <v>3408206340.8010001</v>
+      </c>
+      <c r="F12" s="20">
+        <v>33638</v>
+      </c>
+      <c r="G12" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E12/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F12)</f>
-        <v>37572.92613963395</v>
+        <v>36883.79885212017</v>
       </c>
       <c r="H12" s="8">
-        <f t="shared" si="0"/>
-        <v>10.534039020540032</v>
+        <f>LN(G12)</f>
+        <v>10.515527678117433</v>
       </c>
       <c r="I12" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J12" s="8">
-        <f t="shared" si="1"/>
-        <v>11.481120919934959</v>
+        <f>LN(C12)</f>
+        <v>11.220023257959742</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>322</v>
+        <v>309</v>
       </c>
       <c r="C13" s="19">
-        <v>131664.94</v>
+        <v>66070.73</v>
       </c>
       <c r="D13" s="15">
-        <v>0</v>
+        <v>0.4090515614942401</v>
       </c>
       <c r="E13">
-        <v>3334593535</v>
+        <v>1763633082.14856</v>
       </c>
       <c r="F13">
-        <v>19901</v>
-      </c>
-      <c r="G13" s="23">
+        <v>42994</v>
+      </c>
+      <c r="G13" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E13/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F13)</f>
-        <v>51966.74412229177</v>
+        <v>23423.022489202867</v>
       </c>
       <c r="H13" s="8">
-        <f t="shared" si="0"/>
-        <v>10.85835925686334</v>
+        <f>LN(G13)</f>
+        <v>10.061474684725773</v>
       </c>
       <c r="I13" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J13" s="8">
-        <f t="shared" si="1"/>
-        <v>11.78801564120511</v>
+        <f>LN(C13)</f>
+        <v>11.098481113850436</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>350</v>
+        <v>310</v>
       </c>
       <c r="C14" s="19">
-        <v>77173.179999999993</v>
+        <v>46691.18</v>
       </c>
       <c r="D14" s="15">
         <v>0</v>
       </c>
       <c r="E14">
-        <v>1966649200.72945</v>
+        <v>154360176</v>
       </c>
       <c r="F14">
-        <v>18356</v>
-      </c>
-      <c r="G14" s="23">
+        <v>2304</v>
+      </c>
+      <c r="G14" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E14/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F14)</f>
-        <v>38372.302475809345</v>
+        <v>29221.714306405374</v>
       </c>
       <c r="H14" s="8">
-        <f t="shared" si="0"/>
-        <v>10.55509118862879</v>
+        <f>LN(G14)</f>
+        <v>10.282667352523003</v>
       </c>
       <c r="I14" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J14" s="8">
-        <f t="shared" si="1"/>
-        <v>11.253807266325841</v>
+        <f>LN(C14)</f>
+        <v>10.75131056072337</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="C15" s="19">
-        <v>86513.02</v>
+        <v>65978.06</v>
       </c>
       <c r="D15" s="15">
-        <v>0.1205471526572444</v>
+        <v>8.4275672371638147E-2</v>
       </c>
       <c r="E15">
-        <v>3548280190.2389002</v>
+        <v>797400506</v>
       </c>
       <c r="F15">
-        <v>45538</v>
-      </c>
-      <c r="G15" s="23">
+        <v>11229</v>
+      </c>
+      <c r="G15" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E15/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F15)</f>
-        <v>31797.76055179978</v>
+        <v>30118.21074843104</v>
       </c>
       <c r="H15" s="8">
-        <f t="shared" si="0"/>
-        <v>10.367151143389082</v>
+        <f>LN(G15)</f>
+        <v>10.312885276046782</v>
       </c>
       <c r="I15" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J15" s="8">
-        <f t="shared" si="1"/>
-        <v>11.36805020182415</v>
+        <f>LN(C15)</f>
+        <v>11.097077541500951</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>354</v>
+        <v>312</v>
       </c>
       <c r="C16" s="19">
-        <v>90360.68</v>
+        <v>43564.07</v>
       </c>
       <c r="D16" s="15">
-        <v>0.22267534116153603</v>
+        <v>0.5042573320719016</v>
       </c>
       <c r="E16">
-        <v>5574661088</v>
-      </c>
-      <c r="F16">
-        <v>63031</v>
-      </c>
-      <c r="G16" s="23">
+        <v>1512923307.3832099</v>
+      </c>
+      <c r="F16" s="20">
+        <v>29942</v>
+      </c>
+      <c r="G16" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E16/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F16)</f>
-        <v>34165.672303187246</v>
+        <v>25545.510000382921</v>
       </c>
       <c r="H16" s="8">
-        <f t="shared" si="0"/>
-        <v>10.438976685147631</v>
+        <f>LN(G16)</f>
+        <v>10.148216846348651</v>
       </c>
       <c r="I16" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J16" s="8">
-        <f t="shared" si="1"/>
-        <v>11.411564496007363</v>
+        <f>LN(C16)</f>
+        <v>10.681988007025614</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>332</v>
+        <v>313</v>
       </c>
       <c r="C17" s="19">
-        <v>91410.82</v>
+        <v>53852.46</v>
       </c>
       <c r="D17" s="15">
-        <v>0</v>
+        <v>0.75820207040818155</v>
       </c>
       <c r="E17">
-        <v>5614957192.4309101</v>
+        <v>1892226542</v>
       </c>
       <c r="F17">
-        <v>53332</v>
-      </c>
-      <c r="G17" s="23">
+        <v>54409</v>
+      </c>
+      <c r="G17" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E17/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F17)</f>
-        <v>37954.650567036479</v>
+        <v>22029.473284641641</v>
       </c>
       <c r="H17" s="8">
-        <f t="shared" si="0"/>
-        <v>10.544147319901743</v>
+        <f>LN(G17)</f>
+        <v>10.000136530506554</v>
       </c>
       <c r="I17" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J17" s="8">
-        <f t="shared" si="1"/>
-        <v>11.423119131179776</v>
+        <f>LN(C17)</f>
+        <v>10.894003363992377</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>17</v>
+        <v>64</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C18" s="19">
-        <v>87410.67</v>
+        <v>78436.89</v>
       </c>
       <c r="D18" s="15">
-        <v>0.25343592833800727</v>
+        <v>5.3610100927552813E-2</v>
       </c>
       <c r="E18">
-        <v>4228655447.0969</v>
+        <v>1732124198.8775499</v>
       </c>
       <c r="F18">
-        <v>41233</v>
-      </c>
-      <c r="G18" s="23">
+        <v>23629</v>
+      </c>
+      <c r="G18" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E18/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F18)</f>
-        <v>37340.861127430435</v>
+        <v>30629.949149522356</v>
       </c>
       <c r="H18" s="8">
-        <f t="shared" si="0"/>
-        <v>10.527843478624932</v>
+        <f>LN(G18)</f>
+        <v>10.329733539672729</v>
       </c>
       <c r="I18" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J18" s="8">
-        <f t="shared" si="1"/>
-        <v>11.378372636572042</v>
+        <f>LN(C18)</f>
+        <v>11.27004963138557</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>341</v>
+        <v>315</v>
       </c>
       <c r="C19" s="19">
-        <v>72339.740000000005</v>
+        <v>46865.31</v>
       </c>
       <c r="D19" s="15">
-        <v>0.46219012568571627</v>
+        <v>0.243556256468385</v>
       </c>
       <c r="E19">
-        <v>947789398</v>
+        <v>1480662744</v>
       </c>
       <c r="F19">
-        <v>14280</v>
-      </c>
-      <c r="G19" s="23">
+        <v>21088</v>
+      </c>
+      <c r="G19" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E19/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F19)</f>
-        <v>29199.620287127032</v>
+        <v>29939.831021853097</v>
       </c>
       <c r="H19" s="8">
-        <f t="shared" si="0"/>
-        <v>10.281910984306309</v>
+        <f>LN(G19)</f>
+        <v>10.306945014065011</v>
       </c>
       <c r="I19" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J19" s="8">
-        <f t="shared" si="1"/>
-        <v>11.189128911360841</v>
+        <f>LN(C19)</f>
+        <v>10.755033021903188</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>306</v>
+        <v>316</v>
       </c>
       <c r="C20" s="19">
-        <v>68284.210000000006</v>
+        <v>87410.67</v>
       </c>
       <c r="D20" s="15">
-        <v>0.4069716831378975</v>
+        <v>0.25343592833800727</v>
       </c>
       <c r="E20">
-        <v>3965235780.5862598</v>
+        <v>4199545587.0969</v>
       </c>
       <c r="F20">
-        <v>72088</v>
-      </c>
-      <c r="G20" s="23">
+        <v>41233</v>
+      </c>
+      <c r="G20" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E20/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F20)</f>
-        <v>26642.200895884856</v>
+        <v>37001.891711706936</v>
       </c>
       <c r="H20" s="8">
-        <f t="shared" si="0"/>
-        <v>10.190251737453687</v>
+        <f>LN(G20)</f>
+        <v>10.518724317662834</v>
       </c>
       <c r="I20" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J20" s="8">
-        <f t="shared" si="1"/>
-        <v>11.131433832886929</v>
+        <f>LN(C20)</f>
+        <v>11.378372636572042</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="C21" s="19">
-        <v>70766.63</v>
+        <v>37170.33</v>
       </c>
       <c r="D21" s="15">
-        <v>0.23929847892943229</v>
+        <v>0.68962585034013602</v>
       </c>
       <c r="E21">
-        <v>1280582613.6588299</v>
+        <v>913888258.70661795</v>
       </c>
       <c r="F21">
-        <v>22576</v>
-      </c>
-      <c r="G21" s="23">
+        <v>20731</v>
+      </c>
+      <c r="G21" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E21/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F21)</f>
-        <v>27028.681837922304</v>
+        <v>24106.718918689858</v>
       </c>
       <c r="H21" s="8">
-        <f t="shared" si="0"/>
-        <v>10.204653871448818</v>
+        <f>LN(G21)</f>
+        <v>10.090245873929748</v>
       </c>
       <c r="I21" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J21" s="8">
-        <f t="shared" si="1"/>
-        <v>11.167142840888388</v>
+        <f>LN(C21)</f>
+        <v>10.523266141379409</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="C22" s="19">
-        <v>93915.78</v>
+        <v>61942.46</v>
       </c>
       <c r="D22" s="15">
-        <v>0</v>
+        <v>0.99935555146381883</v>
       </c>
       <c r="E22">
-        <v>3863916690.1880798</v>
-      </c>
-      <c r="F22">
-        <v>35533</v>
-      </c>
-      <c r="G22" s="23">
+        <v>715963426.428491</v>
+      </c>
+      <c r="F22" s="20">
+        <v>22613</v>
+      </c>
+      <c r="G22" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E22/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F22)</f>
-        <v>38732.826126004817</v>
+        <v>21333.831545903959</v>
       </c>
       <c r="H22" s="8">
-        <f t="shared" si="0"/>
-        <v>10.564442739792524</v>
+        <f>LN(G22)</f>
+        <v>9.968049427115254</v>
       </c>
       <c r="I22" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J22" s="8">
-        <f t="shared" si="1"/>
-        <v>11.450153702195557</v>
+        <f>LN(C22)</f>
+        <v>11.033961168592592</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>22</v>
+        <v>77</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>338</v>
+        <v>319</v>
       </c>
       <c r="C23" s="19">
-        <v>107915.53</v>
+        <v>70548.97</v>
       </c>
       <c r="D23" s="15">
-        <v>6.2987511337472962E-2</v>
+        <v>1.7550092368907203E-2</v>
       </c>
       <c r="E23">
-        <v>10349284631.224199</v>
+        <v>5709652228.8214197</v>
       </c>
       <c r="F23">
-        <v>71192</v>
-      </c>
-      <c r="G23" s="23">
+        <v>56563</v>
+      </c>
+      <c r="G23" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E23/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F23)</f>
-        <v>46974.528794062608</v>
+        <v>36799.665469189124</v>
       </c>
       <c r="H23" s="8">
-        <f t="shared" si="0"/>
-        <v>10.757360793237478</v>
+        <f>LN(G23)</f>
+        <v>10.513244033604538</v>
       </c>
       <c r="I23" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J23" s="8">
-        <f t="shared" si="1"/>
-        <v>11.589104070453772</v>
+        <f>LN(C23)</f>
+        <v>11.164062357599615</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="C24" s="19">
-        <v>56531.19</v>
+        <v>128066.04</v>
       </c>
       <c r="D24" s="15">
-        <v>0.45625403858580266</v>
+        <v>0</v>
       </c>
       <c r="E24">
-        <v>3039736669.3952899</v>
+        <v>1712590142</v>
       </c>
       <c r="F24">
-        <v>56153</v>
-      </c>
-      <c r="G24" s="23">
+        <v>11558</v>
+      </c>
+      <c r="G24" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E24/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F24)</f>
-        <v>26445.916053649053</v>
+        <v>47342.95555435821</v>
       </c>
       <c r="H24" s="8">
-        <f t="shared" si="0"/>
-        <v>10.182857022856609</v>
+        <f>LN(G24)</f>
+        <v>10.765173313615096</v>
       </c>
       <c r="I24" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J24" s="8">
-        <f t="shared" si="1"/>
-        <v>10.942547800217275</v>
+        <f>LN(C24)</f>
+        <v>11.760301347351763</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>24</v>
+        <v>68</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>372</v>
+        <v>321</v>
       </c>
       <c r="C25" s="19">
-        <v>141208.35</v>
+        <v>31396.83</v>
       </c>
       <c r="D25" s="15">
-        <v>1.2781809275355716E-2</v>
+        <v>0.9463662850342649</v>
       </c>
       <c r="E25">
-        <v>16462631666.2216</v>
+        <v>569159118</v>
       </c>
       <c r="F25">
-        <v>88164</v>
-      </c>
-      <c r="G25" s="23">
+        <v>23195</v>
+      </c>
+      <c r="G25" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E25/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F25)</f>
-        <v>56279.602685850004</v>
+        <v>19743.626250217741</v>
       </c>
       <c r="H25" s="8">
-        <f t="shared" si="0"/>
-        <v>10.938087451605858</v>
+        <f>LN(G25)</f>
+        <v>9.8905859967355134</v>
       </c>
       <c r="I25" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J25" s="8">
-        <f t="shared" si="1"/>
-        <v>11.857991738270153</v>
+        <f>LN(C25)</f>
+        <v>10.354462211385991</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>303</v>
+        <v>322</v>
       </c>
       <c r="C26" s="19">
-        <v>47532.57</v>
+        <v>131664.94</v>
       </c>
       <c r="D26" s="15">
-        <v>0.49213417981088892</v>
+        <v>0</v>
       </c>
       <c r="E26">
-        <v>4743250985.9707403</v>
+        <v>3279025819</v>
       </c>
       <c r="F26">
-        <v>97452</v>
-      </c>
-      <c r="G26" s="23">
+        <v>19901</v>
+      </c>
+      <c r="G26" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E26/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F26)</f>
-        <v>25217.321836287192</v>
+        <v>51047.103159049242</v>
       </c>
       <c r="H26" s="8">
-        <f t="shared" si="0"/>
-        <v>10.135286411821737</v>
+        <f>LN(G26)</f>
+        <v>10.840504076812307</v>
       </c>
       <c r="I26" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J26" s="8">
-        <f t="shared" si="1"/>
-        <v>10.769170439259247</v>
+        <f>LN(C26)</f>
+        <v>11.78801564120511</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>368</v>
+        <v>323</v>
       </c>
       <c r="C27" s="19">
-        <v>38641.730000000003</v>
+        <v>20239.66</v>
       </c>
       <c r="D27" s="15">
-        <v>0.64332013996443527</v>
+        <v>0.9668874172185431</v>
       </c>
       <c r="E27">
-        <v>532283575.13797301</v>
-      </c>
-      <c r="F27">
-        <v>15096</v>
-      </c>
-      <c r="G27" s="23">
+        <v>98064092</v>
+      </c>
+      <c r="F27" s="20">
+        <v>2345</v>
+      </c>
+      <c r="G27" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E27/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F27)</f>
-        <v>22199.448052026695</v>
+        <v>23601.145340074137</v>
       </c>
       <c r="H27" s="8">
-        <f t="shared" si="0"/>
-        <v>10.007822705029973</v>
+        <f>LN(G27)</f>
+        <v>10.069050521195166</v>
       </c>
       <c r="I27" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J27" s="8">
-        <f t="shared" si="1"/>
-        <v>10.562088059580935</v>
+        <f>LN(C27)</f>
+        <v>9.915399324841335</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>27</v>
+        <v>63</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="C28" s="19">
-        <v>37170.33</v>
+        <v>63701.67</v>
       </c>
       <c r="D28" s="15">
-        <v>0.68962585034013602</v>
+        <v>0.91780475467880629</v>
       </c>
       <c r="E28">
-        <v>934575156.70661795</v>
+        <v>1248469892.1224699</v>
       </c>
       <c r="F28">
-        <v>20731</v>
-      </c>
-      <c r="G28" s="23">
+        <v>36081</v>
+      </c>
+      <c r="G28" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E28/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F28)</f>
-        <v>24409.202414274449</v>
+        <v>21990.19407686243</v>
       </c>
       <c r="H28" s="8">
-        <f t="shared" si="0"/>
-        <v>10.102715488304817</v>
+        <f>LN(G28)</f>
+        <v>9.9983519091971012</v>
       </c>
       <c r="I28" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J28" s="8">
-        <f t="shared" si="1"/>
-        <v>10.523266141379409</v>
+        <f>LN(C28)</f>
+        <v>11.061966057857108</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>346</v>
+        <v>325</v>
       </c>
       <c r="C29" s="19">
-        <v>111332.42</v>
+        <v>96218.19</v>
       </c>
       <c r="D29" s="15">
-        <v>0.1626522885638102</v>
+        <v>0.20226304353960325</v>
       </c>
       <c r="E29">
-        <v>22690599560.388</v>
+        <v>2920911652</v>
       </c>
       <c r="F29">
-        <v>68165</v>
-      </c>
-      <c r="G29" s="23">
+        <v>36732</v>
+      </c>
+      <c r="G29" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E29/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F29)</f>
-        <v>89163.375199745555</v>
+        <v>32017.225190364356</v>
       </c>
       <c r="H29" s="8">
-        <f t="shared" si="0"/>
-        <v>11.39822564232105</v>
+        <f>LN(G29)</f>
+        <v>10.374029324156165</v>
       </c>
       <c r="I29" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J29" s="8">
-        <f t="shared" si="1"/>
-        <v>11.620275779664263</v>
+        <f>LN(C29)</f>
+        <v>11.474373704018522</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>349</v>
+        <v>326</v>
       </c>
       <c r="C30" s="19">
-        <v>42220.59</v>
+        <v>50075.11</v>
       </c>
       <c r="D30" s="15">
-        <v>0.6732482611944588</v>
+        <v>0.40599455040871935</v>
       </c>
       <c r="E30">
-        <v>1255679042.0029199</v>
+        <v>1493820786</v>
       </c>
       <c r="F30">
-        <v>33958</v>
-      </c>
-      <c r="G30" s="23">
+        <v>25181</v>
+      </c>
+      <c r="G30" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E30/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F30)</f>
-        <v>22585.886688312239</v>
+        <v>27508.79933842567</v>
       </c>
       <c r="H30" s="8">
-        <f t="shared" si="0"/>
-        <v>10.025080507371724</v>
+        <f>LN(G30)</f>
+        <v>10.222261208416031</v>
       </c>
       <c r="I30" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J30" s="8">
-        <f t="shared" si="1"/>
-        <v>10.650663295724376</v>
+        <f>LN(C30)</f>
+        <v>10.821279357236548</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>360</v>
+        <v>327</v>
       </c>
       <c r="C31" s="19">
-        <v>54569.47</v>
+        <v>37961.58</v>
       </c>
       <c r="D31" s="15">
-        <v>0.61087690303785769</v>
+        <v>0.51663436179339706</v>
       </c>
       <c r="E31">
-        <v>2214326519.5912199</v>
+        <v>1143447176</v>
       </c>
       <c r="F31">
-        <v>69884</v>
-      </c>
-      <c r="G31" s="23">
+        <v>29143</v>
+      </c>
+      <c r="G31" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E31/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F31)</f>
-        <v>21395.261608846413</v>
+        <v>23024.620121628654</v>
       </c>
       <c r="H31" s="8">
-        <f t="shared" si="0"/>
-        <v>9.9709247563455197</v>
+        <f>LN(G31)</f>
+        <v>10.044319362469649</v>
       </c>
       <c r="I31" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J31" s="8">
-        <f t="shared" si="1"/>
-        <v>10.90722984783698</v>
+        <f>LN(C31)</f>
+        <v>10.544329874618462</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="C32" s="19">
-        <v>80267.06</v>
+        <v>65810.570000000007</v>
       </c>
       <c r="D32" s="15">
-        <v>0.31566472104530235</v>
+        <v>5.2857285329610051E-3</v>
       </c>
       <c r="E32">
-        <v>3355586836.6333699</v>
+        <v>617721898.44498003</v>
       </c>
       <c r="F32">
-        <v>33446</v>
-      </c>
-      <c r="G32" s="23">
+        <v>8927</v>
+      </c>
+      <c r="G32" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E32/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F32)</f>
-        <v>36839.869799365384</v>
+        <v>29712.918550559625</v>
       </c>
       <c r="H32" s="8">
-        <f t="shared" si="0"/>
-        <v>10.514335956143817</v>
+        <f>LN(G32)</f>
+        <v>10.29933719825193</v>
       </c>
       <c r="I32" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J32" s="8">
-        <f t="shared" si="1"/>
-        <v>11.293114604068913</v>
+        <f>LN(C32)</f>
+        <v>11.094535742710331</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>362</v>
+        <v>329</v>
       </c>
       <c r="C33" s="19">
-        <v>119470.67</v>
+        <v>70766.63</v>
       </c>
       <c r="D33" s="15">
-        <v>0</v>
+        <v>0.23929847892943229</v>
       </c>
       <c r="E33">
-        <v>60869319139.509003</v>
+        <v>1294621431.9169199</v>
       </c>
       <c r="F33">
-        <v>42550</v>
-      </c>
-      <c r="G33" s="23">
+        <v>22576</v>
+      </c>
+      <c r="G33" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E33/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F33)</f>
-        <v>336136.41478346387</v>
+        <v>27067.181052027881</v>
       </c>
       <c r="H33" s="8">
-        <f t="shared" si="0"/>
-        <v>12.725272352930469</v>
+        <f>LN(G33)</f>
+        <v>10.206077241686344</v>
       </c>
       <c r="I33" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J33" s="8">
-        <f t="shared" si="1"/>
-        <v>11.690826180897997</v>
+        <f>LN(C33)</f>
+        <v>11.167142840888388</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>345</v>
+        <v>330</v>
       </c>
       <c r="C34" s="19">
-        <v>118169.58</v>
+        <v>56531.19</v>
       </c>
       <c r="D34" s="15">
-        <v>0</v>
+        <v>0.45625403858580266</v>
       </c>
       <c r="E34">
-        <v>7669949196.5560703</v>
+        <v>3008336717.9130502</v>
       </c>
       <c r="F34">
-        <v>30482</v>
-      </c>
-      <c r="G34" s="23">
+        <v>56153</v>
+      </c>
+      <c r="G34" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E34/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F34)</f>
-        <v>70880.939275753539</v>
+        <v>26225.352406803588</v>
       </c>
       <c r="H34" s="8">
-        <f t="shared" ref="H34:H65" si="2">LN(G34)</f>
-        <v>11.168756836824253</v>
+        <f>LN(G34)</f>
+        <v>10.174481870993223</v>
       </c>
       <c r="I34" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J34" s="8">
-        <f t="shared" ref="J34:J65" si="3">LN(C34)</f>
-        <v>11.67987599042517</v>
+        <f>LN(C34)</f>
+        <v>10.942547800217275</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>300</v>
+        <v>331</v>
       </c>
       <c r="C35" s="19">
-        <v>45340.34</v>
+        <v>69838.12</v>
       </c>
       <c r="D35" s="15">
-        <v>0.21713462922966162</v>
+        <v>9.919880499728409E-2</v>
       </c>
       <c r="E35">
-        <v>1398865114</v>
-      </c>
-      <c r="F35" s="20">
-        <v>13885</v>
-      </c>
-      <c r="G35" s="23">
+        <v>3580926386</v>
+      </c>
+      <c r="F35">
+        <v>30599</v>
+      </c>
+      <c r="G35" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E35/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F35)</f>
-        <v>36933.920282844025</v>
+        <v>40390.190953429395</v>
       </c>
       <c r="H35" s="8">
-        <f t="shared" si="2"/>
-        <v>10.516885656635699</v>
+        <f>LN(G35)</f>
+        <v>10.606342236286551</v>
       </c>
       <c r="I35" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J35" s="8">
-        <f t="shared" si="3"/>
-        <v>10.721952422930624</v>
+        <f>LN(C35)</f>
+        <v>11.153935271479922</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>315</v>
+        <v>332</v>
       </c>
       <c r="C36" s="19">
-        <v>46865.31</v>
+        <v>91410.82</v>
       </c>
       <c r="D36" s="15">
-        <v>0.243556256468385</v>
+        <v>0</v>
       </c>
       <c r="E36">
-        <v>1457390874</v>
+        <v>5581578444.4309101</v>
       </c>
       <c r="F36">
-        <v>21088</v>
-      </c>
-      <c r="G36" s="23">
+        <v>53332</v>
+      </c>
+      <c r="G36" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E36/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F36)</f>
-        <v>29815.704776268387</v>
+        <v>37628.741390449475</v>
       </c>
       <c r="H36" s="8">
-        <f t="shared" si="2"/>
-        <v>10.302790539589695</v>
+        <f>LN(G36)</f>
+        <v>10.535523436056275</v>
       </c>
       <c r="I36" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J36" s="8">
-        <f t="shared" si="3"/>
-        <v>10.755033021903188</v>
+        <f>LN(C36)</f>
+        <v>11.423119131179776</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>353</v>
+        <v>333</v>
       </c>
       <c r="C37" s="19">
-        <v>27756.76</v>
+        <v>96869.59</v>
       </c>
       <c r="D37" s="15">
-        <v>1</v>
+        <v>0.37648764113518463</v>
       </c>
       <c r="E37">
-        <v>420233996</v>
+        <v>2737263835.1213899</v>
       </c>
       <c r="F37">
-        <v>6937</v>
-      </c>
-      <c r="G37" s="23">
+        <v>26649</v>
+      </c>
+      <c r="G37" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E37/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F37)</f>
-        <v>27896.157753317995</v>
+        <v>37195.277638474487</v>
       </c>
       <c r="H37" s="8">
-        <f t="shared" si="2"/>
-        <v>10.236244243391045</v>
+        <f>LN(G37)</f>
+        <v>10.523937087000714</v>
       </c>
       <c r="I37" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J37" s="8">
-        <f t="shared" si="3"/>
-        <v>10.231234693111643</v>
+        <f>LN(C37)</f>
+        <v>11.481120919934959</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>323</v>
+        <v>334</v>
       </c>
       <c r="C38" s="19">
-        <v>20239.66</v>
+        <v>64745.87</v>
       </c>
       <c r="D38" s="15">
-        <v>0.9668874172185431</v>
+        <v>0.62879263444235201</v>
       </c>
       <c r="E38">
-        <v>108407276</v>
-      </c>
-      <c r="F38" s="20">
-        <v>2345</v>
-      </c>
-      <c r="G38" s="23">
+        <v>1817501210</v>
+      </c>
+      <c r="F38">
+        <v>18417</v>
+      </c>
+      <c r="G38" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E38/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F38)</f>
-        <v>24667.517972028039</v>
+        <v>36295.793737221873</v>
       </c>
       <c r="H38" s="8">
-        <f t="shared" si="2"/>
-        <v>10.113242595302173</v>
+        <f>LN(G38)</f>
+        <v>10.499457138531254</v>
       </c>
       <c r="I38" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J38" s="8">
-        <f t="shared" si="3"/>
-        <v>9.915399324841335</v>
+        <f>LN(C38)</f>
+        <v>11.078225193743728</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>326</v>
+        <v>335</v>
       </c>
       <c r="C39" s="19">
-        <v>50075.11</v>
+        <v>105498.97</v>
       </c>
       <c r="D39" s="15">
-        <v>0.40599455040871935</v>
+        <v>0</v>
       </c>
       <c r="E39">
-        <v>1473809152</v>
+        <v>20162247693.400501</v>
       </c>
       <c r="F39">
-        <v>25181</v>
-      </c>
-      <c r="G39" s="23">
+        <v>102827</v>
+      </c>
+      <c r="G39" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E39/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F39)</f>
-        <v>27434.904285828678</v>
+        <v>58037.017575257349</v>
       </c>
       <c r="H39" s="8">
-        <f t="shared" si="2"/>
-        <v>10.219571360725507</v>
+        <f>LN(G39)</f>
+        <v>10.968836319999982</v>
       </c>
       <c r="I39" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J39" s="8">
-        <f t="shared" si="3"/>
-        <v>10.821279357236548</v>
+        <f>LN(C39)</f>
+        <v>11.566456468817425</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C40" s="19">
-        <v>64745.87</v>
+        <v>137914.1</v>
       </c>
       <c r="D40" s="15">
-        <v>0.62879263444235201</v>
+        <v>0</v>
       </c>
       <c r="E40">
-        <v>1816301258</v>
+        <v>20527671967</v>
       </c>
       <c r="F40">
-        <v>18417</v>
-      </c>
-      <c r="G40" s="23">
+        <v>67987</v>
+      </c>
+      <c r="G40" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E40/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F40)</f>
-        <v>36455.662983952301</v>
+        <v>81667.377664387357</v>
       </c>
       <c r="H40" s="8">
-        <f t="shared" si="2"/>
-        <v>10.503852088440606</v>
+        <f>LN(G40)</f>
+        <v>11.310409906915396</v>
       </c>
       <c r="I40" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J40" s="8">
-        <f t="shared" si="3"/>
-        <v>11.078225193743728</v>
+        <f>LN(C40)</f>
+        <v>11.834386306560223</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>365</v>
+        <v>337</v>
       </c>
       <c r="C41" s="19">
-        <v>35737.18</v>
+        <v>92490.48</v>
       </c>
       <c r="D41" s="15">
-        <v>0.67443141575509558</v>
+        <v>0</v>
       </c>
       <c r="E41">
-        <v>474204750</v>
+        <v>5369096809.7778797</v>
       </c>
       <c r="F41">
-        <v>12313</v>
-      </c>
-      <c r="G41" s="23">
+        <v>41651</v>
+      </c>
+      <c r="G41" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E41/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F41)</f>
-        <v>22931.286849221273</v>
+        <v>43042.007059603377</v>
       </c>
       <c r="H41" s="8">
-        <f t="shared" si="2"/>
-        <v>10.04025749504572</v>
+        <f>LN(G41)</f>
+        <v>10.669931826174137</v>
       </c>
       <c r="I41" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J41" s="8">
-        <f t="shared" si="3"/>
-        <v>10.483946882410695</v>
+        <f>LN(C41)</f>
+        <v>11.434860999285082</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="C42" s="19">
-        <v>69838.12</v>
+        <v>107915.53</v>
       </c>
       <c r="D42" s="15">
-        <v>9.919880499728409E-2</v>
+        <v>6.2987511337472962E-2</v>
       </c>
       <c r="E42">
-        <v>3571513320</v>
+        <v>10310558879.0436</v>
       </c>
       <c r="F42">
-        <v>30599</v>
-      </c>
-      <c r="G42" s="23">
+        <v>71192</v>
+      </c>
+      <c r="G42" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E42/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F42)</f>
-        <v>40527.941485496318</v>
+        <v>46596.005990919053</v>
       </c>
       <c r="H42" s="8">
-        <f t="shared" si="2"/>
-        <v>10.60974692843604</v>
+        <f>LN(G42)</f>
+        <v>10.74927010809119</v>
       </c>
       <c r="I42" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J42" s="8">
-        <f t="shared" si="3"/>
-        <v>11.153935271479922</v>
+        <f>LN(C42)</f>
+        <v>11.589104070453772</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>373</v>
+        <v>339</v>
       </c>
       <c r="C43" s="19">
-        <v>39802.04</v>
+        <v>80267.06</v>
       </c>
       <c r="D43" s="15">
-        <v>0.64528147389969293</v>
+        <v>0.31566472104530235</v>
       </c>
       <c r="E43">
-        <v>1087817372</v>
+        <v>3323989868.12713</v>
       </c>
       <c r="F43">
-        <v>23801</v>
-      </c>
-      <c r="G43" s="23">
+        <v>33446</v>
+      </c>
+      <c r="G43" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E43/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F43)</f>
-        <v>24549.52273060118</v>
+        <v>36451.545917665055</v>
       </c>
       <c r="H43" s="8">
-        <f t="shared" si="2"/>
-        <v>10.108447692324985</v>
+        <f>LN(G43)</f>
+        <v>10.503739148544712</v>
       </c>
       <c r="I43" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J43" s="8">
-        <f t="shared" si="3"/>
-        <v>10.591673446240378</v>
+        <f>LN(C43)</f>
+        <v>11.293114604068913</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>361</v>
+        <v>340</v>
       </c>
       <c r="C44" s="19">
-        <v>44027.92</v>
+        <v>79959.789999999994</v>
       </c>
       <c r="D44" s="15">
-        <v>0.46788089900131552</v>
+        <v>0.21836337373610501</v>
       </c>
       <c r="E44">
-        <v>2059404538</v>
+        <v>1233066664.6865699</v>
       </c>
       <c r="F44">
-        <v>53588</v>
-      </c>
-      <c r="G44" s="23">
+        <v>14854</v>
+      </c>
+      <c r="G44" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E44/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F44)</f>
-        <v>22912.792503483804</v>
+        <v>32796.948617168018</v>
       </c>
       <c r="H44" s="8">
-        <f t="shared" si="2"/>
-        <v>10.039450658175969</v>
+        <f>LN(G44)</f>
+        <v>10.39809076008029</v>
       </c>
       <c r="I44" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J44" s="8">
-        <f t="shared" si="3"/>
-        <v>10.692579257116103</v>
+        <f>LN(C44)</f>
+        <v>11.289279162297731</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>312</v>
+        <v>341</v>
       </c>
       <c r="C45" s="19">
-        <v>43564.07</v>
+        <v>72339.740000000005</v>
       </c>
       <c r="D45" s="15">
-        <v>0.5042573320719016</v>
+        <v>0.46219012568571627</v>
       </c>
       <c r="E45">
-        <v>1517860263.90818</v>
-      </c>
-      <c r="F45" s="20">
-        <v>29942</v>
-      </c>
-      <c r="G45" s="23">
+        <v>938028756</v>
+      </c>
+      <c r="F45">
+        <v>14280</v>
+      </c>
+      <c r="G45" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E45/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F45)</f>
-        <v>25671.969854932602</v>
+        <v>28929.657220091533</v>
       </c>
       <c r="H45" s="8">
-        <f t="shared" si="2"/>
-        <v>10.153155008549856</v>
+        <f>LN(G45)</f>
+        <v>10.27262254930308</v>
       </c>
       <c r="I45" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J45" s="8">
-        <f t="shared" si="3"/>
-        <v>10.681988007025614</v>
+        <f>LN(C45)</f>
+        <v>11.189128911360841</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>304</v>
+        <v>342</v>
       </c>
       <c r="C46" s="19">
-        <v>57862.6</v>
+        <v>70807.509999999995</v>
       </c>
       <c r="D46" s="15">
-        <v>0</v>
+        <v>0.31365052393089776</v>
       </c>
       <c r="E46">
-        <v>554922436</v>
+        <v>1495655536.28953</v>
       </c>
       <c r="F46" s="20">
-        <v>9024</v>
-      </c>
-      <c r="G46" s="23">
+        <v>20873</v>
+      </c>
+      <c r="G46" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E46/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F46)</f>
-        <v>28102.129033629561</v>
+        <v>30261.621849919888</v>
       </c>
       <c r="H46" s="8">
-        <f t="shared" si="2"/>
-        <v>10.243600618773051</v>
+        <f>LN(G46)</f>
+        <v>10.317635583061387</v>
       </c>
       <c r="I46" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J46" s="8">
-        <f t="shared" si="3"/>
-        <v>10.965826513573072</v>
+        <f>LN(C46)</f>
+        <v>11.167720347502749</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47">
-        <v>46</v>
+        <v>74</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>358</v>
+        <v>343</v>
       </c>
       <c r="C47" s="19">
-        <v>40515.019999999997</v>
+        <v>115423.08</v>
       </c>
       <c r="D47" s="15">
-        <v>0.63666666666666671</v>
+        <v>0.82639038007300836</v>
       </c>
       <c r="E47">
-        <v>886136027.60169101</v>
+        <v>1603307654</v>
       </c>
       <c r="F47">
-        <v>27551</v>
-      </c>
-      <c r="G47" s="23">
+        <v>19059</v>
+      </c>
+      <c r="G47" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E47/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F47)</f>
-        <v>21502.752098546414</v>
+        <v>33044.948814713651</v>
       </c>
       <c r="H47" s="8">
-        <f t="shared" si="2"/>
-        <v>9.9759362105074203</v>
+        <f>LN(G47)</f>
+        <v>10.405623998946284</v>
       </c>
       <c r="I47" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J47" s="8">
-        <f t="shared" si="3"/>
-        <v>10.609428048539034</v>
+        <f>LN(C47)</f>
+        <v>11.656359613058802</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>310</v>
+        <v>344</v>
       </c>
       <c r="C48" s="19">
-        <v>46691.18</v>
+        <v>124208.23</v>
       </c>
       <c r="D48" s="15">
         <v>0</v>
       </c>
       <c r="E48">
-        <v>154979128</v>
+        <v>133150650239.28799</v>
       </c>
       <c r="F48">
-        <v>2304</v>
-      </c>
-      <c r="G48" s="23">
+        <v>107331</v>
+      </c>
+      <c r="G48" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E48/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F48)</f>
-        <v>29400.644134449816</v>
+        <v>291198.03299102857</v>
       </c>
       <c r="H48" s="8">
-        <f t="shared" si="2"/>
-        <v>10.288771862421795</v>
+        <f>LN(G48)</f>
+        <v>12.581758840443353</v>
       </c>
       <c r="I48" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J48" s="8">
-        <f t="shared" si="3"/>
-        <v>10.75131056072337</v>
+        <f>LN(C48)</f>
+        <v>11.729714710376324</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>311</v>
+        <v>345</v>
       </c>
       <c r="C49" s="19">
-        <v>65978.06</v>
+        <v>118169.58</v>
       </c>
       <c r="D49" s="15">
-        <v>8.4275672371638147E-2</v>
+        <v>0</v>
       </c>
       <c r="E49">
-        <v>801655546</v>
+        <v>7925645746.0561705</v>
       </c>
       <c r="F49">
-        <v>11229</v>
-      </c>
-      <c r="G49" s="23">
+        <v>30482</v>
+      </c>
+      <c r="G49" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E49/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F49)</f>
-        <v>30329.058382254443</v>
+        <v>72308.501796823009</v>
       </c>
       <c r="H49" s="8">
-        <f t="shared" si="2"/>
-        <v>10.319861554445815</v>
+        <f>LN(G49)</f>
+        <v>11.188696991784431</v>
       </c>
       <c r="I49" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J49" s="8">
-        <f t="shared" si="3"/>
-        <v>11.097077541500951</v>
+        <f>LN(C49)</f>
+        <v>11.67987599042517</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>357</v>
+        <v>346</v>
       </c>
       <c r="C50" s="19">
-        <v>48744.81</v>
+        <v>111332.42</v>
       </c>
       <c r="D50" s="15">
-        <v>0.64146228359439406</v>
+        <v>0.1626522885638102</v>
       </c>
       <c r="E50">
-        <v>1467654352.7150199</v>
+        <v>24735880873.030602</v>
       </c>
       <c r="F50">
-        <v>36635</v>
-      </c>
-      <c r="G50" s="23">
+        <v>68165</v>
+      </c>
+      <c r="G50" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E50/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F50)</f>
-        <v>23279.813424141306</v>
+        <v>95272.696519273115</v>
       </c>
       <c r="H50" s="8">
-        <f t="shared" si="2"/>
-        <v>10.055341887386339</v>
+        <f>LN(G50)</f>
+        <v>11.464498548270813</v>
       </c>
       <c r="I50" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J50" s="8">
-        <f t="shared" si="3"/>
-        <v>10.7943540092201</v>
+        <f>LN(C50)</f>
+        <v>11.620275779664263</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="C51" s="19">
-        <v>62475.37</v>
+        <v>55496.94</v>
       </c>
       <c r="D51" s="15">
-        <v>0.48020527859237538</v>
+        <v>0.44576877234803336</v>
       </c>
       <c r="E51">
-        <v>463034211.20127797</v>
-      </c>
-      <c r="F51">
-        <v>6744</v>
-      </c>
-      <c r="G51" s="23">
+        <v>1731024519.1602099</v>
+      </c>
+      <c r="F51" s="20">
+        <v>40065</v>
+      </c>
+      <c r="G51" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E51/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F51)</f>
-        <v>29714.16889171064</v>
+        <v>23910.773442368569</v>
       </c>
       <c r="H51" s="8">
-        <f t="shared" si="2"/>
-        <v>10.299379278091445</v>
+        <f>LN(G51)</f>
+        <v>10.082084407999805</v>
       </c>
       <c r="I51" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J51" s="8">
-        <f t="shared" si="3"/>
-        <v>11.042527678054563</v>
+        <f>LN(C51)</f>
+        <v>10.924083163079393</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>359</v>
+        <v>348</v>
       </c>
       <c r="C52" s="19">
-        <v>39340</v>
+        <v>145659.34</v>
       </c>
       <c r="D52" s="15">
         <v>0</v>
       </c>
       <c r="E52">
-        <v>632440233.59475005</v>
+        <v>7388587780.5430002</v>
       </c>
       <c r="F52">
-        <v>12854</v>
-      </c>
-      <c r="G52" s="23">
+        <v>36014</v>
+      </c>
+      <c r="G52" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E52/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F52)</f>
-        <v>25336.376691141828</v>
+        <v>60063.835317721801</v>
       </c>
       <c r="H52" s="8">
-        <f t="shared" si="2"/>
-        <v>10.139996455930094</v>
+        <f>LN(G52)</f>
+        <v>11.003163197602406</v>
       </c>
       <c r="I52" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J52" s="8">
-        <f t="shared" si="3"/>
-        <v>10.579997091943049</v>
+        <f>LN(C52)</f>
+        <v>11.88902588666182</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>318</v>
+        <v>349</v>
       </c>
       <c r="C53" s="19">
-        <v>61942.46</v>
+        <v>42220.59</v>
       </c>
       <c r="D53" s="15">
-        <v>0.99935555146381883</v>
+        <v>0.6732482611944588</v>
       </c>
       <c r="E53">
-        <v>717220175.04682505</v>
-      </c>
-      <c r="F53" s="20">
-        <v>22613</v>
-      </c>
-      <c r="G53" s="23">
+        <v>1201042675.8569601</v>
+      </c>
+      <c r="F53">
+        <v>33958</v>
+      </c>
+      <c r="G53" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E53/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F53)</f>
-        <v>21402.330607194534</v>
+        <v>22161.325440894147</v>
       </c>
       <c r="H53" s="8">
-        <f t="shared" si="2"/>
-        <v>9.9712551019582687</v>
+        <f>LN(G53)</f>
+        <v>10.006103951387253</v>
       </c>
       <c r="I53" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J53" s="8">
-        <f t="shared" si="3"/>
-        <v>11.033961168592592</v>
+        <f>LN(C53)</f>
+        <v>10.650663295724376</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54">
-        <v>53</v>
+        <v>13</v>
       </c>
       <c r="B54" s="13" t="s">
-        <v>370</v>
+        <v>350</v>
       </c>
       <c r="C54" s="19">
-        <v>54430.28</v>
+        <v>77173.179999999993</v>
       </c>
       <c r="D54" s="15">
-        <v>0.89373276126264178</v>
+        <v>0</v>
       </c>
       <c r="E54">
-        <v>894063121.09593594</v>
+        <v>1952269532.3166299</v>
       </c>
       <c r="F54">
-        <v>24549</v>
-      </c>
-      <c r="G54" s="23">
+        <v>18356</v>
+      </c>
+      <c r="G54" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E54/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F54)</f>
-        <v>22460.363485927017</v>
+        <v>38007.949373216659</v>
       </c>
       <c r="H54" s="8">
-        <f t="shared" si="2"/>
-        <v>10.019507411862593</v>
+        <f>LN(G54)</f>
+        <v>10.54555061086252</v>
       </c>
       <c r="I54" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J54" s="8">
-        <f t="shared" si="3"/>
-        <v>10.904675895636951</v>
+        <f>LN(C54)</f>
+        <v>11.253807266325841</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55">
-        <v>54</v>
+        <v>10</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>224</v>
+        <v>351</v>
       </c>
       <c r="C55" s="19">
-        <v>17638.89</v>
+        <v>110554.42</v>
       </c>
       <c r="D55" s="15">
-        <v>1</v>
-      </c>
-      <c r="E55" s="21">
-        <v>88633152</v>
-      </c>
-      <c r="F55">
-        <v>7518</v>
-      </c>
-      <c r="G55" s="23">
+        <v>0.3766284625225178</v>
+      </c>
+      <c r="E55">
+        <v>4694332680</v>
+      </c>
+      <c r="F55" s="20">
+        <v>39840</v>
+      </c>
+      <c r="G55" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E55/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F55)</f>
-        <v>16918.600631610832</v>
+        <v>40569.238765925045</v>
       </c>
       <c r="H55" s="8">
-        <f t="shared" si="2"/>
-        <v>9.7361689247524286</v>
+        <f>LN(G55)</f>
+        <v>10.610765392552064</v>
       </c>
       <c r="I55" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J55" s="8">
-        <f t="shared" si="3"/>
-        <v>9.7778614024108421</v>
+        <f>LN(C55)</f>
+        <v>11.613263167394976</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="B56" s="13" t="s">
-        <v>328</v>
+        <v>353</v>
       </c>
       <c r="C56" s="19">
-        <v>65810.570000000007</v>
+        <v>27756.76</v>
       </c>
       <c r="D56" s="15">
-        <v>5.2857285329610051E-3</v>
+        <v>1</v>
       </c>
       <c r="E56">
-        <v>555427497.29508102</v>
+        <v>429050113</v>
       </c>
       <c r="F56">
-        <v>8927</v>
-      </c>
-      <c r="G56" s="23">
+        <v>6937</v>
+      </c>
+      <c r="G56" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E56/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F56)</f>
-        <v>28265.201255865053</v>
+        <v>28072.72370444463</v>
       </c>
       <c r="H56" s="8">
-        <f t="shared" si="2"/>
-        <v>10.249386689404758</v>
+        <f>LN(G56)</f>
+        <v>10.242553697225866</v>
       </c>
       <c r="I56" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J56" s="8">
-        <f t="shared" si="3"/>
-        <v>11.094535742710331</v>
+        <f>LN(C56)</f>
+        <v>10.231234693111643</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="B57" s="13" t="s">
-        <v>325</v>
+        <v>352</v>
       </c>
       <c r="C57" s="19">
-        <v>96218.19</v>
+        <v>83115.61</v>
       </c>
       <c r="D57" s="15">
-        <v>0.20226304353960325</v>
+        <v>0</v>
       </c>
       <c r="E57">
-        <v>2929880472</v>
-      </c>
-      <c r="F57">
-        <v>36732</v>
-      </c>
-      <c r="G57" s="23">
+        <v>1704801477.6924701</v>
+      </c>
+      <c r="F57" s="20">
+        <v>14394</v>
+      </c>
+      <c r="G57" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E57/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F57)</f>
-        <v>32212.795694695851</v>
+        <v>40705.120844688761</v>
       </c>
       <c r="H57" s="8">
-        <f t="shared" si="2"/>
-        <v>10.380119034420106</v>
+        <f>LN(G57)</f>
+        <v>10.614109182795927</v>
       </c>
       <c r="I57" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J57" s="8">
-        <f t="shared" si="3"/>
-        <v>11.474373704018522</v>
+        <f>LN(C57)</f>
+        <v>11.327987809171407</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="B58" s="13" t="s">
-        <v>299</v>
+        <v>354</v>
       </c>
       <c r="C58" s="19">
-        <v>67012.2</v>
+        <v>90360.68</v>
       </c>
       <c r="D58" s="15">
-        <v>9.270216962524655E-2</v>
+        <v>0.22267534116153603</v>
       </c>
       <c r="E58">
-        <v>994396260.73109198</v>
+        <v>5529760840.5041904</v>
       </c>
       <c r="F58">
-        <v>13414</v>
-      </c>
-      <c r="G58" s="23">
+        <v>63031</v>
+      </c>
+      <c r="G58" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E58/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F58)</f>
-        <v>30945.488356178976</v>
+        <v>33850.238898617732</v>
       </c>
       <c r="H58" s="8">
-        <f t="shared" si="2"/>
-        <v>10.339982495473366</v>
+        <f>LN(G58)</f>
+        <v>10.429701335881772</v>
       </c>
       <c r="I58" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J58" s="8">
-        <f t="shared" si="3"/>
-        <v>11.112629971349051</v>
+        <f>LN(C58)</f>
+        <v>11.411564496007363</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B59" s="13" t="s">
-        <v>309</v>
+        <v>355</v>
       </c>
       <c r="C59" s="19">
-        <v>66070.73</v>
+        <v>62475.37</v>
       </c>
       <c r="D59" s="15">
-        <v>0.4090515614942401</v>
+        <v>0.48020527859237538</v>
       </c>
       <c r="E59">
-        <v>1780426102.36166</v>
+        <v>448315198.45997101</v>
       </c>
       <c r="F59">
-        <v>42994</v>
-      </c>
-      <c r="G59" s="23">
+        <v>6744</v>
+      </c>
+      <c r="G59" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E59/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F59)</f>
-        <v>23583.45093437202</v>
+        <v>29105.534056873323</v>
       </c>
       <c r="H59" s="8">
-        <f t="shared" si="2"/>
-        <v>10.068300513441423</v>
+        <f>LN(G59)</f>
+        <v>10.278683608854559</v>
       </c>
       <c r="I59" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J59" s="8">
-        <f t="shared" si="3"/>
-        <v>11.098481113850436</v>
+        <f>LN(C59)</f>
+        <v>11.042527678054563</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B60" s="13" t="s">
-        <v>340</v>
+        <v>224</v>
       </c>
       <c r="C60" s="19">
-        <v>79959.789999999994</v>
+        <v>17638.89</v>
       </c>
       <c r="D60" s="15">
-        <v>0.21836337373610501</v>
+        <v>1</v>
       </c>
       <c r="E60">
-        <v>1238142773.8199301</v>
+        <v>93486026</v>
       </c>
       <c r="F60">
-        <v>14854</v>
-      </c>
-      <c r="G60" s="23">
+        <v>7518</v>
+      </c>
+      <c r="G60" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E60/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F60)</f>
-        <v>33020.648368242088</v>
+        <v>17041.8466115189</v>
       </c>
       <c r="H60" s="8">
-        <f t="shared" si="2"/>
-        <v>10.404888352903454</v>
+        <f>LN(G60)</f>
+        <v>9.7434271637323793</v>
       </c>
       <c r="I60" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J60" s="8">
-        <f t="shared" si="3"/>
-        <v>11.289279162297731</v>
+        <f>LN(C60)</f>
+        <v>9.7778614024108421</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="B61" s="13" t="s">
-        <v>308</v>
+        <v>356</v>
       </c>
       <c r="C61" s="19">
-        <v>74609.509999999995</v>
+        <v>60915.74</v>
       </c>
       <c r="D61" s="15">
-        <v>7.6879710402943446E-2</v>
+        <v>0.29557057596893649</v>
       </c>
       <c r="E61">
-        <v>3425149601.8145499</v>
-      </c>
-      <c r="F61" s="20">
-        <v>33638</v>
-      </c>
-      <c r="G61" s="23">
+        <v>3894460410</v>
+      </c>
+      <c r="F61">
+        <v>54173</v>
+      </c>
+      <c r="G61" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E61/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F61)</f>
-        <v>37176.317367303091</v>
+        <v>30313.92284181363</v>
       </c>
       <c r="H61" s="8">
-        <f t="shared" si="2"/>
-        <v>10.523427207615159</v>
+        <f>LN(G61)</f>
+        <v>10.319362385689612</v>
       </c>
       <c r="I61" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J61" s="8">
-        <f t="shared" si="3"/>
-        <v>11.220023257959742</v>
+        <f>LN(C61)</f>
+        <v>11.017246876789907</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="B62" s="13" t="s">
-        <v>347</v>
+        <v>357</v>
       </c>
       <c r="C62" s="19">
-        <v>55496.94</v>
+        <v>48744.81</v>
       </c>
       <c r="D62" s="15">
-        <v>0.44576877234803336</v>
+        <v>0.64146228359439406</v>
       </c>
       <c r="E62">
-        <v>1744139059.0571401</v>
-      </c>
-      <c r="F62" s="20">
-        <v>40065</v>
-      </c>
-      <c r="G62" s="23">
+        <v>1449606528.7150199</v>
+      </c>
+      <c r="F62">
+        <v>36635</v>
+      </c>
+      <c r="G62" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E62/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F62)</f>
-        <v>24060.832944099311</v>
+        <v>23098.991078811232</v>
       </c>
       <c r="H62" s="8">
-        <f t="shared" si="2"/>
-        <v>10.088340608384929</v>
+        <f>LN(G62)</f>
+        <v>10.047544219314112</v>
       </c>
       <c r="I62" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J62" s="8">
-        <f t="shared" si="3"/>
-        <v>10.924083163079393</v>
+        <f>LN(C62)</f>
+        <v>10.7943540092201</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="B63" s="13" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
       <c r="C63" s="19">
-        <v>75895.23</v>
+        <v>40515.019999999997</v>
       </c>
       <c r="D63" s="15">
-        <v>0.75171251495052738</v>
+        <v>0.63666666666666671</v>
       </c>
       <c r="E63">
-        <v>943420954</v>
+        <v>879604365.20338202</v>
       </c>
       <c r="F63">
-        <v>17901</v>
-      </c>
-      <c r="G63" s="23">
+        <v>27551</v>
+      </c>
+      <c r="G63" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E63/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F63)</f>
-        <v>26123.946772669988</v>
+        <v>21392.947461675496</v>
       </c>
       <c r="H63" s="8">
-        <f t="shared" si="2"/>
-        <v>10.170607673532722</v>
+        <f>LN(G63)</f>
+        <v>9.9708165888281854</v>
       </c>
       <c r="I63" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J63" s="8">
-        <f t="shared" si="3"/>
-        <v>11.237109115559036</v>
+        <f>LN(C63)</f>
+        <v>10.609428048539034</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="B64" s="13" t="s">
-        <v>324</v>
+        <v>359</v>
       </c>
       <c r="C64" s="19">
-        <v>63701.67</v>
+        <v>39340</v>
       </c>
       <c r="D64" s="15">
-        <v>0.91780475467880629</v>
+        <v>0</v>
       </c>
       <c r="E64">
-        <v>1259700999.6398001</v>
+        <v>639138915.49758601</v>
       </c>
       <c r="F64">
-        <v>36081</v>
-      </c>
-      <c r="G64" s="23">
+        <v>12854</v>
+      </c>
+      <c r="G64" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E64/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F64)</f>
-        <v>22121.425218013243</v>
+        <v>25365.695783051095</v>
       </c>
       <c r="H64" s="8">
-        <f t="shared" si="2"/>
-        <v>10.00430188475476</v>
+        <f>LN(G64)</f>
+        <v>10.14115298045647</v>
       </c>
       <c r="I64" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J64" s="8">
-        <f t="shared" si="3"/>
-        <v>11.061966057857108</v>
+        <f>LN(C64)</f>
+        <v>10.579997091943049</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65">
-        <v>64</v>
+        <v>30</v>
       </c>
       <c r="B65" s="13" t="s">
-        <v>314</v>
+        <v>360</v>
       </c>
       <c r="C65" s="19">
-        <v>78436.89</v>
+        <v>54569.47</v>
       </c>
       <c r="D65" s="15">
-        <v>5.3610100927552813E-2</v>
+        <v>0.61087690303785769</v>
       </c>
       <c r="E65">
-        <v>1740504096.6638999</v>
+        <v>2274481373.9562602</v>
       </c>
       <c r="F65">
-        <v>23629</v>
-      </c>
-      <c r="G65" s="23">
+        <v>69884</v>
+      </c>
+      <c r="G65" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E65/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F65)</f>
-        <v>30839.386071080582</v>
+        <v>21531.3778851553</v>
       </c>
       <c r="H65" s="8">
-        <f t="shared" si="2"/>
-        <v>10.33654792057512</v>
+        <f>LN(G65)</f>
+        <v>9.9772665866921741</v>
       </c>
       <c r="I65" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J65" s="8">
-        <f t="shared" si="3"/>
-        <v>11.27004963138557</v>
+        <f>LN(C65)</f>
+        <v>10.90722984783698</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="B66" s="13" t="s">
-        <v>369</v>
+        <v>361</v>
       </c>
       <c r="C66" s="19">
-        <v>73122.880000000005</v>
+        <v>44027.92</v>
       </c>
       <c r="D66" s="15">
-        <v>0.66009149783138255</v>
+        <v>0.46788089900131552</v>
       </c>
       <c r="E66">
-        <v>1662849170</v>
+        <v>1991331096</v>
       </c>
       <c r="F66">
-        <v>31942</v>
-      </c>
-      <c r="G66" s="23">
+        <v>53588</v>
+      </c>
+      <c r="G66" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E66/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F66)</f>
-        <v>25979.10434398982</v>
+        <v>22561.254143677575</v>
       </c>
       <c r="H66" s="8">
-        <f t="shared" ref="H66:H97" si="4">LN(G66)</f>
-        <v>10.165047814803138</v>
+        <f>LN(G66)</f>
+        <v>10.023989295541917</v>
       </c>
       <c r="I66" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J66" s="8">
-        <f t="shared" ref="J66:J78" si="5">LN(C66)</f>
-        <v>11.199896592660906</v>
+        <f>LN(C66)</f>
+        <v>10.692579257116103</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="B67" s="13" t="s">
-        <v>313</v>
+        <v>362</v>
       </c>
       <c r="C67" s="19">
-        <v>53852.46</v>
+        <v>119470.67</v>
       </c>
       <c r="D67" s="15">
-        <v>0.75820207040818155</v>
+        <v>0</v>
       </c>
       <c r="E67">
-        <v>1912350686</v>
+        <v>62800380163.2892</v>
       </c>
       <c r="F67">
-        <v>54409</v>
-      </c>
-      <c r="G67" s="23">
+        <v>42550</v>
+      </c>
+      <c r="G67" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E67/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F67)</f>
-        <v>22174.199046455957</v>
+        <v>343737.45416588429</v>
       </c>
       <c r="H67" s="8">
-        <f t="shared" si="4"/>
-        <v>10.006684686861682</v>
+        <f>LN(G67)</f>
+        <v>12.747633430324914</v>
       </c>
       <c r="I67" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J67" s="8">
-        <f t="shared" si="5"/>
-        <v>10.894003363992377</v>
+        <f>LN(C67)</f>
+        <v>11.690826180897997</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>67</v>
+        <v>3</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C68" s="19">
-        <v>38273.449999999997</v>
+        <v>70066.83</v>
       </c>
       <c r="D68" s="15">
-        <v>0.67517792694033119</v>
+        <v>0</v>
       </c>
       <c r="E68">
-        <v>627711081.28356099</v>
+        <v>6281493234</v>
       </c>
       <c r="F68">
-        <v>28144</v>
-      </c>
-      <c r="G68" s="23">
+        <v>56344</v>
+      </c>
+      <c r="G68" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E68/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F68)</f>
-        <v>19284.269238772584</v>
+        <v>39152.847674295335</v>
       </c>
       <c r="H68" s="8">
-        <f t="shared" si="4"/>
-        <v>9.8670449771980433</v>
+        <f>LN(G68)</f>
+        <v>10.575228436303597</v>
       </c>
       <c r="I68" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J68" s="8">
-        <f t="shared" si="5"/>
-        <v>10.552511723298306</v>
+        <f>LN(C68)</f>
+        <v>11.157204779867387</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B69" s="13" t="s">
-        <v>321</v>
+        <v>364</v>
       </c>
       <c r="C69" s="19">
-        <v>31396.83</v>
+        <v>68129.460000000006</v>
       </c>
       <c r="D69" s="15">
-        <v>0.9463662850342649</v>
+        <v>0.75599441452224214</v>
       </c>
       <c r="E69">
-        <v>586459514</v>
+        <v>1271715507.2748699</v>
       </c>
       <c r="F69">
-        <v>23195</v>
-      </c>
-      <c r="G69" s="23">
+        <v>24851</v>
+      </c>
+      <c r="G69" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E69/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F69)</f>
-        <v>19954.842458564995</v>
+        <v>25689.527629406824</v>
       </c>
       <c r="H69" s="8">
-        <f t="shared" si="4"/>
-        <v>9.9012271226165414</v>
+        <f>LN(G69)</f>
+        <v>10.153838702601552</v>
       </c>
       <c r="I69" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J69" s="8">
-        <f t="shared" si="5"/>
-        <v>10.354462211385991</v>
+        <f>LN(C69)</f>
+        <v>11.129164997712525</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70">
-        <v>69</v>
+        <v>40</v>
       </c>
       <c r="B70" s="13" t="s">
-        <v>327</v>
+        <v>365</v>
       </c>
       <c r="C70" s="19">
-        <v>37961.58</v>
+        <v>35737.18</v>
       </c>
       <c r="D70" s="15">
-        <v>0.51663436179339706</v>
+        <v>0.67443141575509558</v>
       </c>
       <c r="E70">
-        <v>1151954740</v>
+        <v>476450594</v>
       </c>
       <c r="F70">
-        <v>29143</v>
-      </c>
-      <c r="G70" s="23">
+        <v>12313</v>
+      </c>
+      <c r="G70" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E70/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F70)</f>
-        <v>23159.692639054912</v>
+        <v>22903.892920391241</v>
       </c>
       <c r="H70" s="8">
-        <f t="shared" si="4"/>
-        <v>10.050168660400894</v>
+        <f>LN(G70)</f>
+        <v>10.039062171618195</v>
       </c>
       <c r="I70" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J70" s="8">
-        <f t="shared" si="5"/>
-        <v>10.544329874618462</v>
+        <f>LN(C70)</f>
+        <v>10.483946882410695</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="B71" s="13" t="s">
-        <v>301</v>
+        <v>366</v>
       </c>
       <c r="C71" s="19">
-        <v>82235.360000000001</v>
+        <v>75895.23</v>
       </c>
       <c r="D71" s="15">
-        <v>0.30595162781643875</v>
+        <v>0.75171251495052738</v>
       </c>
       <c r="E71">
-        <v>2591607528.0592399</v>
+        <v>938670954</v>
       </c>
       <c r="F71">
-        <v>42007</v>
-      </c>
-      <c r="G71" s="23">
+        <v>17901</v>
+      </c>
+      <c r="G71" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E71/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F71)</f>
-        <v>28147.262748444457</v>
+        <v>25971.507541389929</v>
       </c>
       <c r="H71" s="8">
-        <f t="shared" si="4"/>
-        <v>10.245205390773993</v>
+        <f>LN(G71)</f>
+        <v>10.164755352313156</v>
       </c>
       <c r="I71" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J71" s="8">
-        <f t="shared" si="5"/>
-        <v>11.317340658863849</v>
+        <f>LN(C71)</f>
+        <v>11.237109115559036</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B72" s="13" t="s">
-        <v>302</v>
+        <v>367</v>
       </c>
       <c r="C72" s="19">
-        <v>47170.47</v>
+        <v>38273.449999999997</v>
       </c>
       <c r="D72" s="15">
-        <v>0.59438923303177504</v>
+        <v>0.67517792694033119</v>
       </c>
       <c r="E72">
-        <v>1852067815</v>
+        <v>615677087.28356099</v>
       </c>
       <c r="F72">
-        <v>43779</v>
-      </c>
-      <c r="G72" s="23">
+        <v>28144</v>
+      </c>
+      <c r="G72" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E72/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F72)</f>
-        <v>23784.578298603978</v>
+        <v>19149.374105201947</v>
       </c>
       <c r="H72" s="8">
-        <f t="shared" si="4"/>
-        <v>10.076792678988964</v>
+        <f>LN(G72)</f>
+        <v>9.8600253102731994</v>
       </c>
       <c r="I72" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J72" s="8">
-        <f t="shared" si="5"/>
-        <v>10.761523340188811</v>
+        <f>LN(C72)</f>
+        <v>10.552511723298306</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="B73" s="13" t="s">
-        <v>307</v>
+        <v>368</v>
       </c>
       <c r="C73" s="19">
-        <v>132096.54</v>
+        <v>38641.730000000003</v>
       </c>
       <c r="D73" s="15">
-        <v>0</v>
+        <v>0.64332013996443527</v>
       </c>
       <c r="E73">
-        <v>2206100566</v>
+        <v>530526289.57916802</v>
       </c>
       <c r="F73">
-        <v>19521</v>
-      </c>
-      <c r="G73" s="23">
+        <v>15096</v>
+      </c>
+      <c r="G73" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E73/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F73)</f>
-        <v>39693.579417037537</v>
+        <v>22111.104164635675</v>
       </c>
       <c r="H73" s="8">
-        <f t="shared" si="4"/>
-        <v>10.588944726065433</v>
+        <f>LN(G73)</f>
+        <v>10.003835212208156</v>
       </c>
       <c r="I73" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J73" s="8">
-        <f t="shared" si="5"/>
-        <v>11.791288297888816</v>
+        <f>LN(C73)</f>
+        <v>10.562088059580935</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B74" s="13" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C74" s="19">
-        <v>68129.460000000006</v>
+        <v>73122.880000000005</v>
       </c>
       <c r="D74" s="15">
-        <v>0.75599441452224214</v>
+        <v>0.66009149783138255</v>
       </c>
       <c r="E74">
-        <v>1274341977.2748699</v>
+        <v>1661667786.2862899</v>
       </c>
       <c r="F74">
-        <v>24851</v>
-      </c>
-      <c r="G74" s="23">
+        <v>31942</v>
+      </c>
+      <c r="G74" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E74/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F74)</f>
-        <v>25803.809518441463</v>
+        <v>25878.781371777695</v>
       </c>
       <c r="H74" s="8">
-        <f t="shared" si="4"/>
-        <v>10.158277415763216</v>
+        <f>LN(G74)</f>
+        <v>10.161178659862349</v>
       </c>
       <c r="I74" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J74" s="8">
-        <f t="shared" si="5"/>
-        <v>11.129164997712525</v>
+        <f>LN(C74)</f>
+        <v>11.199896592660906</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="B75" s="13" t="s">
-        <v>343</v>
+        <v>370</v>
       </c>
       <c r="C75" s="19">
-        <v>115423.08</v>
+        <v>54430.28</v>
       </c>
       <c r="D75" s="15">
-        <v>0.82639038007300836</v>
+        <v>0.89373276126264178</v>
       </c>
       <c r="E75">
-        <v>1628720074</v>
+        <v>885370209.09593594</v>
       </c>
       <c r="F75">
-        <v>19059</v>
-      </c>
-      <c r="G75" s="23">
+        <v>24549</v>
+      </c>
+      <c r="G75" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E75/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F75)</f>
-        <v>33493.728091490651</v>
+        <v>22316.907319687853</v>
       </c>
       <c r="H75" s="8">
-        <f t="shared" si="4"/>
-        <v>10.419113479135557</v>
+        <f>LN(G75)</f>
+        <v>10.013099845948908</v>
       </c>
       <c r="I75" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J75" s="8">
-        <f t="shared" si="5"/>
-        <v>11.656359613058802</v>
+        <f>LN(C75)</f>
+        <v>10.904675895636951</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="B76" s="13" t="s">
-        <v>342</v>
+        <v>371</v>
       </c>
       <c r="C76" s="19">
-        <v>70807.509999999995</v>
+        <v>70823.37</v>
       </c>
       <c r="D76" s="15">
-        <v>0.31365052393089776</v>
+        <v>5.750628873732528E-2</v>
       </c>
       <c r="E76">
-        <v>1505913598.3160801</v>
-      </c>
-      <c r="F76" s="20">
-        <v>20873</v>
-      </c>
-      <c r="G76" s="23">
+        <v>5277053447</v>
+      </c>
+      <c r="F76">
+        <v>78373</v>
+      </c>
+      <c r="G76" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E76/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F76)</f>
-        <v>30498.922206284326</v>
+        <v>29296.706529185285</v>
       </c>
       <c r="H76" s="8">
-        <f t="shared" si="4"/>
-        <v>10.325446624472244</v>
+        <f>LN(G76)</f>
+        <v>10.285230383539966</v>
       </c>
       <c r="I76" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J76" s="8">
-        <f t="shared" si="5"/>
-        <v>11.167720347502749</v>
+        <f>LN(C76)</f>
+        <v>11.167944309961589</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77">
-        <v>76</v>
+        <v>24</v>
       </c>
       <c r="B77" s="13" t="s">
-        <v>352</v>
+        <v>372</v>
       </c>
       <c r="C77" s="19">
-        <v>83115.61</v>
+        <v>141208.35</v>
       </c>
       <c r="D77" s="15">
-        <v>0</v>
+        <v>1.2781809275355716E-2</v>
       </c>
       <c r="E77">
-        <v>1697988043.6924701</v>
-      </c>
-      <c r="F77" s="20">
-        <v>14394</v>
-      </c>
-      <c r="G77" s="23">
+        <v>16519483419.702299</v>
+      </c>
+      <c r="F77">
+        <v>88164</v>
+      </c>
+      <c r="G77" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E77/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F77)</f>
-        <v>40808.078102530264</v>
+        <v>56093.318878039361</v>
       </c>
       <c r="H77" s="8">
-        <f t="shared" si="4"/>
-        <v>10.616635333503359</v>
+        <f>LN(G77)</f>
+        <v>10.934771991335566</v>
       </c>
       <c r="I77" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J77" s="8">
-        <f t="shared" si="5"/>
-        <v>11.327987809171407</v>
+        <f>LN(C77)</f>
+        <v>11.857991738270153</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="B78" s="13" t="s">
-        <v>319</v>
+        <v>373</v>
       </c>
       <c r="C78" s="19">
-        <v>70548.97</v>
+        <v>39802.04</v>
       </c>
       <c r="D78" s="15">
-        <v>1.7550092368907203E-2</v>
+        <v>0.64528147389969293</v>
       </c>
       <c r="E78">
-        <v>5719026262</v>
+        <v>1145968560</v>
       </c>
       <c r="F78">
-        <v>56563</v>
-      </c>
-      <c r="G78" s="23">
+        <v>23801</v>
+      </c>
+      <c r="G78" s="22">
         <f>(FACTORS_MUNI!$E$42/FACTORS_MUNI!$C$42)+(E78/SUM(E$2:E$78)*FACTORS_MUNI!$F$42/F78)</f>
-        <v>37015.474976378719</v>
+        <v>25014.096959304734</v>
       </c>
       <c r="H78" s="8">
-        <f t="shared" si="4"/>
-        <v>10.519091346792132</v>
+        <f>LN(G78)</f>
+        <v>10.127194823302856</v>
       </c>
       <c r="I78" s="8">
         <f>FACTORS_MUNI!$K$42</f>
         <v>14.812911489078509</v>
       </c>
       <c r="J78" s="8">
-        <f t="shared" si="5"/>
-        <v>11.164062357599615</v>
+        <f>LN(C78)</f>
+        <v>10.591673446240378</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J78" xr:uid="{00000000-0001-0000-0100-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J78">
-      <sortCondition ref="A1:A78"/>
+      <sortCondition ref="B1:B78"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>